<commit_message>
Add verified Dorchester draw, team sheet and player statistics for 27 October
</commit_message>
<xml_diff>
--- a/Tiverton_Town_SL1_Fixtures_2026-27.xlsx
+++ b/Tiverton_Town_SL1_Fixtures_2026-27.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixtures" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fixtures" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W12"/>
+  <dimension ref="A1:W18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -567,7 +567,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Source: https://www.tivvyarchive.co.uk/season.php?year=2026  |  Updated: sample data current through 2026-10-03</t>
+          <t>Source: https://www.tivvyarchive.co.uk/season.php?year=2026  |  Updated: 2026-10-27 22:28:29 UTC</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>Louis Slough</t>
+          <t>Louie Slough</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
@@ -826,7 +826,7 @@
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>Louis Slough (G 3')</t>
+          <t>Louie Slough (G 3')</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr">
@@ -889,7 +889,11 @@
           <t>Billy Tucker (85')</t>
         </is>
       </c>
-      <c r="T7" s="13" t="n"/>
+      <c r="T7" s="14" t="inlineStr">
+        <is>
+          <t>Caleb Pryce-Hall</t>
+        </is>
+      </c>
       <c r="U7" s="13" t="n"/>
       <c r="V7" s="13" t="n"/>
       <c r="W7" s="13" t="n"/>
@@ -927,22 +931,22 @@
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>Louis Slough</t>
+          <t>Louie Slough</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>Ed Palmer (C)</t>
+          <t>Ed Palmer (C / 63')</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>Asa Hall</t>
+          <t>Asa Hall (56')</t>
         </is>
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>Aaron Wellington</t>
+          <t>Aaron Wellington (63')</t>
         </is>
       </c>
       <c r="K8" s="8" t="inlineStr">
@@ -952,7 +956,7 @@
       </c>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>Finn Roberts</t>
+          <t>Finn Roberts (56')</t>
         </is>
       </c>
       <c r="M8" s="8" t="inlineStr">
@@ -962,7 +966,7 @@
       </c>
       <c r="N8" s="8" t="inlineStr">
         <is>
-          <t>Owen Howe</t>
+          <t>Owen Howe (56')</t>
         </is>
       </c>
       <c r="O8" s="6" t="inlineStr">
@@ -970,29 +974,29 @@
           <t>SUBS:</t>
         </is>
       </c>
-      <c r="P8" s="9" t="inlineStr">
-        <is>
-          <t>Ryan Keates</t>
-        </is>
-      </c>
-      <c r="Q8" s="9" t="inlineStr">
-        <is>
-          <t>Billy Tucker</t>
-        </is>
-      </c>
-      <c r="R8" s="9" t="inlineStr">
-        <is>
-          <t>Aiden Horne</t>
-        </is>
-      </c>
-      <c r="S8" s="9" t="inlineStr">
-        <is>
-          <t>Matt Wood</t>
-        </is>
-      </c>
-      <c r="T8" s="9" t="inlineStr">
-        <is>
-          <t>Caleb Pryce-Hall</t>
+      <c r="P8" s="8" t="inlineStr">
+        <is>
+          <t>Ryan Keates (56')</t>
+        </is>
+      </c>
+      <c r="Q8" s="8" t="inlineStr">
+        <is>
+          <t>Billy Tucker (56')</t>
+        </is>
+      </c>
+      <c r="R8" s="8" t="inlineStr">
+        <is>
+          <t>Aiden Horne (56')</t>
+        </is>
+      </c>
+      <c r="S8" s="8" t="inlineStr">
+        <is>
+          <t>Matt Wood (63')</t>
+        </is>
+      </c>
+      <c r="T8" s="8" t="inlineStr">
+        <is>
+          <t>Caleb Pryce-Hall (63')</t>
         </is>
       </c>
       <c r="U8" s="8" t="n"/>
@@ -1027,7 +1031,7 @@
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>Louis Slough</t>
+          <t>Louie Slough (70')</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
@@ -1042,7 +1046,7 @@
       </c>
       <c r="I9" s="13" t="inlineStr">
         <is>
-          <t>Asa Hall</t>
+          <t>Asa Hall (86')</t>
         </is>
       </c>
       <c r="J9" s="13" t="inlineStr">
@@ -1062,12 +1066,12 @@
       </c>
       <c r="M9" s="13" t="inlineStr">
         <is>
-          <t>Billy Tucker</t>
+          <t>Billy Tucker (67')</t>
         </is>
       </c>
       <c r="N9" s="13" t="inlineStr">
         <is>
-          <t>Owen Howe</t>
+          <t>Owen Howe (86')</t>
         </is>
       </c>
       <c r="O9" s="11" t="inlineStr">
@@ -1075,24 +1079,24 @@
           <t>SUBS:</t>
         </is>
       </c>
-      <c r="P9" s="14" t="inlineStr">
-        <is>
-          <t>Aiden Horne</t>
-        </is>
-      </c>
-      <c r="Q9" s="14" t="inlineStr">
-        <is>
-          <t>Corey Koerner</t>
-        </is>
-      </c>
-      <c r="R9" s="14" t="inlineStr">
-        <is>
-          <t>Aaron Wellington</t>
-        </is>
-      </c>
-      <c r="S9" s="14" t="inlineStr">
-        <is>
-          <t>Ryan Keates</t>
+      <c r="P9" s="13" t="inlineStr">
+        <is>
+          <t>Aiden Horne (67')</t>
+        </is>
+      </c>
+      <c r="Q9" s="13" t="inlineStr">
+        <is>
+          <t>Corey Koerner (70')</t>
+        </is>
+      </c>
+      <c r="R9" s="13" t="inlineStr">
+        <is>
+          <t>Aaron Wellington (86')</t>
+        </is>
+      </c>
+      <c r="S9" s="13" t="inlineStr">
+        <is>
+          <t>Ryan Keates (86')</t>
         </is>
       </c>
       <c r="T9" s="13" t="n"/>
@@ -1128,7 +1132,7 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>Louis Slough</t>
+          <t>Louie Slough</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
@@ -1138,7 +1142,7 @@
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>Ed Palmer (C)</t>
+          <t>Ed Palmer</t>
         </is>
       </c>
       <c r="I10" s="8" t="inlineStr">
@@ -1238,32 +1242,32 @@
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>Louis Slough</t>
+          <t>Ed Palmer (C)</t>
         </is>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>Ed Palmer (C)</t>
+          <t>Louie Slough</t>
         </is>
       </c>
       <c r="I11" s="13" t="inlineStr">
         <is>
+          <t>Ryan Keates (57')</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>Finn Roberts (G 64')</t>
+        </is>
+      </c>
+      <c r="K11" s="13" t="inlineStr">
+        <is>
           <t>Aaron Wellington</t>
         </is>
       </c>
-      <c r="J11" s="13" t="inlineStr">
-        <is>
-          <t>Ryan Keates (57')</t>
-        </is>
-      </c>
-      <c r="K11" s="13" t="inlineStr">
+      <c r="L11" s="13" t="inlineStr">
         <is>
           <t>Jacob Wellington</t>
-        </is>
-      </c>
-      <c r="L11" s="13" t="inlineStr">
-        <is>
-          <t>Finn Roberts (G 64')</t>
         </is>
       </c>
       <c r="M11" s="13" t="inlineStr">
@@ -1338,47 +1342,47 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>Louis Slough</t>
+          <t>Ed Palmer (C)</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Ed Palmer (C)</t>
+          <t>Louie Slough</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
+          <t>Ryan Keates (54')</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
           <t>Josh Bissett</t>
         </is>
       </c>
-      <c r="I12" s="8" t="inlineStr">
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>Finn Roberts (G 38' / 68')</t>
+        </is>
+      </c>
+      <c r="K12" s="8" t="inlineStr">
+        <is>
+          <t>Aaron Wellington (71')</t>
+        </is>
+      </c>
+      <c r="L12" s="8" t="inlineStr">
+        <is>
+          <t>Jacob Wellington</t>
+        </is>
+      </c>
+      <c r="M12" s="8" t="inlineStr">
         <is>
           <t>Owen Howe</t>
         </is>
       </c>
-      <c r="J12" s="8" t="inlineStr">
-        <is>
-          <t>Ryan Keates (54')</t>
-        </is>
-      </c>
-      <c r="K12" s="8" t="inlineStr">
-        <is>
-          <t>Jacob Wellington</t>
-        </is>
-      </c>
-      <c r="L12" s="8" t="inlineStr">
-        <is>
-          <t>Finn Roberts (G 38' / 68')</t>
-        </is>
-      </c>
-      <c r="M12" s="8" t="inlineStr">
+      <c r="N12" s="8" t="inlineStr">
         <is>
           <t>Aiden Horne (G 25')</t>
-        </is>
-      </c>
-      <c r="N12" s="8" t="inlineStr">
-        <is>
-          <t>Aaron Wellington (71')</t>
         </is>
       </c>
       <c r="O12" s="6" t="inlineStr">
@@ -1410,6 +1414,628 @@
       <c r="U12" s="8" t="n"/>
       <c r="V12" s="8" t="n"/>
       <c r="W12" s="8" t="n"/>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>06/10</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>HARTPURY</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>Louis Smith</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>Mason Winter</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>Ed Palmer (C)</t>
+        </is>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>Matt Wood (G 71')</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="inlineStr">
+        <is>
+          <t>Asa Hall</t>
+        </is>
+      </c>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>Ryan Keates (G 47' / 52')</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr">
+        <is>
+          <t>Josh Bissett (87')</t>
+        </is>
+      </c>
+      <c r="K13" s="13" t="inlineStr">
+        <is>
+          <t>Finn Roberts (57')</t>
+        </is>
+      </c>
+      <c r="L13" s="13" t="inlineStr">
+        <is>
+          <t>Jacob Wellington</t>
+        </is>
+      </c>
+      <c r="M13" s="13" t="inlineStr">
+        <is>
+          <t>Owen Howe (G 41' / 90+1')</t>
+        </is>
+      </c>
+      <c r="N13" s="13" t="inlineStr">
+        <is>
+          <t>Aiden Horne (66')</t>
+        </is>
+      </c>
+      <c r="O13" s="11" t="inlineStr">
+        <is>
+          <t>SUBS:</t>
+        </is>
+      </c>
+      <c r="P13" s="13" t="inlineStr">
+        <is>
+          <t>Corey Koerner (57')</t>
+        </is>
+      </c>
+      <c r="Q13" s="13" t="inlineStr">
+        <is>
+          <t>Aaron Wellington (66')</t>
+        </is>
+      </c>
+      <c r="R13" s="13" t="inlineStr">
+        <is>
+          <t>Billy Tucker (87')</t>
+        </is>
+      </c>
+      <c r="S13" s="13" t="inlineStr">
+        <is>
+          <t>Jack Kennell (52')</t>
+        </is>
+      </c>
+      <c r="T13" s="13" t="inlineStr">
+        <is>
+          <t>Louie Slough (90+1')</t>
+        </is>
+      </c>
+      <c r="U13" s="13" t="n"/>
+      <c r="V13" s="13" t="n"/>
+      <c r="W13" s="13" t="n"/>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Shaftesbury</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Louis Smith</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Mason Winter</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Ed Palmer (C / 2G 5', 76')</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Matt Wood</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>Aaron Wellington (89')</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Jack Kennell</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>Asa Hall (65')</t>
+        </is>
+      </c>
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>Corey Koerner</t>
+        </is>
+      </c>
+      <c r="L14" s="8" t="inlineStr">
+        <is>
+          <t>Josh Bissett (G 62' / 78')</t>
+        </is>
+      </c>
+      <c r="M14" s="8" t="inlineStr">
+        <is>
+          <t>Jacob Wellington (85')</t>
+        </is>
+      </c>
+      <c r="N14" s="8" t="inlineStr">
+        <is>
+          <t>Owen Howe (G 36')</t>
+        </is>
+      </c>
+      <c r="O14" s="6" t="inlineStr">
+        <is>
+          <t>SUBS:</t>
+        </is>
+      </c>
+      <c r="P14" s="8" t="inlineStr">
+        <is>
+          <t>Toby Stephens (65')</t>
+        </is>
+      </c>
+      <c r="Q14" s="8" t="inlineStr">
+        <is>
+          <t>Billy Tucker (78')</t>
+        </is>
+      </c>
+      <c r="R14" s="8" t="inlineStr">
+        <is>
+          <t>Finn Roberts (85')</t>
+        </is>
+      </c>
+      <c r="S14" s="8" t="inlineStr">
+        <is>
+          <t>Ryan Keates (89')</t>
+        </is>
+      </c>
+      <c r="T14" s="9" t="inlineStr">
+        <is>
+          <t>Louis Slough</t>
+        </is>
+      </c>
+      <c r="U14" s="8" t="n"/>
+      <c r="V14" s="8" t="n"/>
+      <c r="W14" s="8" t="n"/>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>13/10</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Falmouth Town</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Louis Smith</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>Jack Kennell</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Ed Palmer (C)</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="inlineStr">
+        <is>
+          <t>Matt Wood (65')</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="inlineStr">
+        <is>
+          <t>Aaron Wellington (75')</t>
+        </is>
+      </c>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>Asa Hall (G 11')</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr">
+        <is>
+          <t>Toby Stephens (65')</t>
+        </is>
+      </c>
+      <c r="K15" s="13" t="inlineStr">
+        <is>
+          <t>Corey Koerner</t>
+        </is>
+      </c>
+      <c r="L15" s="13" t="inlineStr">
+        <is>
+          <t>Josh Bissett</t>
+        </is>
+      </c>
+      <c r="M15" s="13" t="inlineStr">
+        <is>
+          <t>Jacob Wellington</t>
+        </is>
+      </c>
+      <c r="N15" s="13" t="inlineStr">
+        <is>
+          <t>Owen Howe</t>
+        </is>
+      </c>
+      <c r="O15" s="11" t="inlineStr">
+        <is>
+          <t>SUBS:</t>
+        </is>
+      </c>
+      <c r="P15" s="13" t="inlineStr">
+        <is>
+          <t>Louis Slough (65')</t>
+        </is>
+      </c>
+      <c r="Q15" s="13" t="inlineStr">
+        <is>
+          <t>Finn Roberts (65')</t>
+        </is>
+      </c>
+      <c r="R15" s="13" t="inlineStr">
+        <is>
+          <t>Aiden Horne (75')</t>
+        </is>
+      </c>
+      <c r="S15" s="13" t="n"/>
+      <c r="T15" s="13" t="n"/>
+      <c r="U15" s="13" t="n"/>
+      <c r="V15" s="13" t="n"/>
+      <c r="W15" s="13" t="n"/>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>17/10</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>PORTLAND UNITED</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Louis Smith</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>Mason Winter</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Ed Palmer (C)</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Louis Slough</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>Jack Kennell (57')</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>Finn Roberts (78')</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>Aaron Wellington (57')</t>
+        </is>
+      </c>
+      <c r="K16" s="8" t="inlineStr">
+        <is>
+          <t>Asa Hall (87')</t>
+        </is>
+      </c>
+      <c r="L16" s="8" t="inlineStr">
+        <is>
+          <t>Jacob Wellington</t>
+        </is>
+      </c>
+      <c r="M16" s="8" t="inlineStr">
+        <is>
+          <t>Josh Bissett</t>
+        </is>
+      </c>
+      <c r="N16" s="8" t="inlineStr">
+        <is>
+          <t>Owen Howe</t>
+        </is>
+      </c>
+      <c r="O16" s="6" t="inlineStr">
+        <is>
+          <t>SUBS:</t>
+        </is>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>Toby Stephens (57')</t>
+        </is>
+      </c>
+      <c r="Q16" s="8" t="inlineStr">
+        <is>
+          <t>Billy Tucker (57')</t>
+        </is>
+      </c>
+      <c r="R16" s="8" t="inlineStr">
+        <is>
+          <t>Matt Wood (87')</t>
+        </is>
+      </c>
+      <c r="S16" s="8" t="inlineStr">
+        <is>
+          <t>Aiden Horne (G 90+1' / 78')</t>
+        </is>
+      </c>
+      <c r="T16" s="9" t="inlineStr">
+        <is>
+          <t>Ryan Keates</t>
+        </is>
+      </c>
+      <c r="U16" s="8" t="n"/>
+      <c r="V16" s="8" t="n"/>
+      <c r="W16" s="8" t="n"/>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>24/10</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Larkhall Athletic</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Louis Smith</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>Mason Winter</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Louie Slough</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>Matt Wood (C)</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="inlineStr">
+        <is>
+          <t>Josh Bissett (3G 2', 28', 64' / 81')</t>
+        </is>
+      </c>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>Asa Hall</t>
+        </is>
+      </c>
+      <c r="J17" s="13" t="inlineStr">
+        <is>
+          <t>Owen Howe</t>
+        </is>
+      </c>
+      <c r="K17" s="13" t="inlineStr">
+        <is>
+          <t>Jacob Wellington (78')</t>
+        </is>
+      </c>
+      <c r="L17" s="13" t="inlineStr">
+        <is>
+          <t>Finn Roberts (90')</t>
+        </is>
+      </c>
+      <c r="M17" s="13" t="inlineStr">
+        <is>
+          <t>Jack Kennell</t>
+        </is>
+      </c>
+      <c r="N17" s="13" t="inlineStr">
+        <is>
+          <t>Aaron Wellington</t>
+        </is>
+      </c>
+      <c r="O17" s="11" t="inlineStr">
+        <is>
+          <t>SUBS:</t>
+        </is>
+      </c>
+      <c r="P17" s="13" t="inlineStr">
+        <is>
+          <t>Tobias Alsop (90')</t>
+        </is>
+      </c>
+      <c r="Q17" s="13" t="inlineStr">
+        <is>
+          <t>Louis Jagger Cane (81')</t>
+        </is>
+      </c>
+      <c r="R17" s="13" t="inlineStr">
+        <is>
+          <t>Toby Stephens (78')</t>
+        </is>
+      </c>
+      <c r="S17" s="14" t="inlineStr">
+        <is>
+          <t>Aiden Horne</t>
+        </is>
+      </c>
+      <c r="T17" s="14" t="inlineStr">
+        <is>
+          <t>Ryan Keates</t>
+        </is>
+      </c>
+      <c r="U17" s="13" t="n"/>
+      <c r="V17" s="13" t="n"/>
+      <c r="W17" s="13" t="n"/>
+    </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>27/10</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>DORCHESTER TOWN</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Louis Smith</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>Mason Winter</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Louie Slough</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Matt Wood (C)</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>Josh Bissett (56')</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Asa Hall</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>Owen Howe (G 90+3')</t>
+        </is>
+      </c>
+      <c r="K18" s="8" t="inlineStr">
+        <is>
+          <t>Jacob Wellington</t>
+        </is>
+      </c>
+      <c r="L18" s="8" t="inlineStr">
+        <is>
+          <t>Finn Roberts (86')</t>
+        </is>
+      </c>
+      <c r="M18" s="8" t="inlineStr">
+        <is>
+          <t>Jack Kennell</t>
+        </is>
+      </c>
+      <c r="N18" s="8" t="inlineStr">
+        <is>
+          <t>Aaron Wellington (81')</t>
+        </is>
+      </c>
+      <c r="O18" s="6" t="inlineStr">
+        <is>
+          <t>SUBS:</t>
+        </is>
+      </c>
+      <c r="P18" s="9" t="inlineStr">
+        <is>
+          <t>Corey Koerner</t>
+        </is>
+      </c>
+      <c r="Q18" s="8" t="inlineStr">
+        <is>
+          <t>Louis Jagger Cane (G 69' / 56')</t>
+        </is>
+      </c>
+      <c r="R18" s="8" t="inlineStr">
+        <is>
+          <t>Tobias Alsop (86')</t>
+        </is>
+      </c>
+      <c r="S18" s="8" t="inlineStr">
+        <is>
+          <t>Toby Stephens (81')</t>
+        </is>
+      </c>
+      <c r="T18" s="9" t="inlineStr">
+        <is>
+          <t>Ryan Keates</t>
+        </is>
+      </c>
+      <c r="U18" s="8" t="n"/>
+      <c r="V18" s="8" t="n"/>
+      <c r="W18" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>